<commit_message>
Remove original task backlink column from Backlog
</commit_message>
<xml_diff>
--- a/plugins/agentic-artefact-project-collaboration/skills/agentic-artefact-project-collaboration/assets/project-plan/Project Timeline Template.xlsx
+++ b/plugins/agentic-artefact-project-collaboration/skills/agentic-artefact-project-collaboration/assets/project-plan/Project Timeline Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="1" r:id="Rf05affaa95b348b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Re28972afd7db40ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="1" r:id="R44dd6cd5169f408b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rc5d0f9ead9ae4911"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1656,7 +1656,6 @@
     <x:col min="6" max="6" width="10.5600004196167" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="25.559999465942383" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12.220000267028809" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -1684,9 +1683,6 @@
       <x:c r="H1" s="28" t="str">
         <x:v>Deliverables</x:v>
       </x:c>
-      <x:c r="I1" s="28" t="str">
-        <x:v>Source task</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" ht="76" customHeight="1">
       <x:c r="A2" s="29"/>
@@ -1697,7 +1693,6 @@
       <x:c r="F2" s="31"/>
       <x:c r="G2" s="29"/>
       <x:c r="H2" s="29"/>
-      <x:c r="I2" s="29"/>
     </x:row>
     <x:row r="3" ht="76" customHeight="1">
       <x:c r="A3" s="29"/>
@@ -1708,7 +1703,6 @@
       <x:c r="F3" s="31"/>
       <x:c r="G3" s="29"/>
       <x:c r="H3" s="29"/>
-      <x:c r="I3" s="29"/>
     </x:row>
     <x:row r="4" ht="76" customHeight="1">
       <x:c r="A4" s="29"/>
@@ -1719,7 +1713,6 @@
       <x:c r="F4" s="31"/>
       <x:c r="G4" s="29"/>
       <x:c r="H4" s="29"/>
-      <x:c r="I4" s="29"/>
     </x:row>
     <x:row r="5" ht="76" customHeight="1">
       <x:c r="A5" s="29"/>
@@ -1730,7 +1723,6 @@
       <x:c r="F5" s="31"/>
       <x:c r="G5" s="29"/>
       <x:c r="H5" s="29"/>
-      <x:c r="I5" s="29"/>
     </x:row>
     <x:row r="6" ht="76" customHeight="1">
       <x:c r="A6" s="29"/>
@@ -1741,7 +1733,6 @@
       <x:c r="F6" s="31"/>
       <x:c r="G6" s="29"/>
       <x:c r="H6" s="29"/>
-      <x:c r="I6" s="29"/>
     </x:row>
     <x:row r="7" ht="76" customHeight="1">
       <x:c r="A7" s="29"/>
@@ -1752,7 +1743,6 @@
       <x:c r="F7" s="31"/>
       <x:c r="G7" s="29"/>
       <x:c r="H7" s="29"/>
-      <x:c r="I7" s="29"/>
     </x:row>
     <x:row r="8" ht="76" customHeight="1">
       <x:c r="A8" s="29"/>
@@ -1763,7 +1753,6 @@
       <x:c r="F8" s="31"/>
       <x:c r="G8" s="29"/>
       <x:c r="H8" s="29"/>
-      <x:c r="I8" s="29"/>
     </x:row>
     <x:row r="9" ht="76" customHeight="1">
       <x:c r="A9" s="29"/>
@@ -1774,7 +1763,6 @@
       <x:c r="F9" s="31"/>
       <x:c r="G9" s="29"/>
       <x:c r="H9" s="29"/>
-      <x:c r="I9" s="29"/>
     </x:row>
     <x:row r="10" ht="76" customHeight="1">
       <x:c r="A10" s="29"/>
@@ -1785,7 +1773,6 @@
       <x:c r="F10" s="31"/>
       <x:c r="G10" s="29"/>
       <x:c r="H10" s="29"/>
-      <x:c r="I10" s="29"/>
     </x:row>
     <x:row r="11" ht="76" customHeight="1">
       <x:c r="A11" s="29"/>
@@ -1796,7 +1783,6 @@
       <x:c r="F11" s="31"/>
       <x:c r="G11" s="29"/>
       <x:c r="H11" s="29"/>
-      <x:c r="I11" s="29"/>
     </x:row>
     <x:row r="12" ht="76" customHeight="1">
       <x:c r="A12" s="29"/>
@@ -1807,7 +1793,6 @@
       <x:c r="F12" s="31"/>
       <x:c r="G12" s="29"/>
       <x:c r="H12" s="29"/>
-      <x:c r="I12" s="29"/>
     </x:row>
     <x:row r="13" ht="76" customHeight="1">
       <x:c r="A13" s="29"/>
@@ -1818,7 +1803,6 @@
       <x:c r="F13" s="31"/>
       <x:c r="G13" s="29"/>
       <x:c r="H13" s="29"/>
-      <x:c r="I13" s="29"/>
     </x:row>
     <x:row r="14" ht="76" customHeight="1">
       <x:c r="A14" s="29"/>
@@ -1829,7 +1813,6 @@
       <x:c r="F14" s="31"/>
       <x:c r="G14" s="29"/>
       <x:c r="H14" s="29"/>
-      <x:c r="I14" s="29"/>
     </x:row>
     <x:row r="15" ht="76" customHeight="1">
       <x:c r="A15" s="29"/>
@@ -1840,7 +1823,6 @@
       <x:c r="F15" s="31"/>
       <x:c r="G15" s="29"/>
       <x:c r="H15" s="29"/>
-      <x:c r="I15" s="29"/>
     </x:row>
     <x:row r="16" ht="76" customHeight="1">
       <x:c r="A16" s="29"/>
@@ -1851,7 +1833,6 @@
       <x:c r="F16" s="31"/>
       <x:c r="G16" s="29"/>
       <x:c r="H16" s="29"/>
-      <x:c r="I16" s="29"/>
     </x:row>
     <x:row r="17" ht="76" customHeight="1">
       <x:c r="A17" s="29"/>
@@ -1862,7 +1843,6 @@
       <x:c r="F17" s="31"/>
       <x:c r="G17" s="29"/>
       <x:c r="H17" s="29"/>
-      <x:c r="I17" s="29"/>
     </x:row>
     <x:row r="18" ht="76" customHeight="1">
       <x:c r="A18" s="29"/>
@@ -1873,7 +1853,6 @@
       <x:c r="F18" s="31"/>
       <x:c r="G18" s="29"/>
       <x:c r="H18" s="29"/>
-      <x:c r="I18" s="29"/>
     </x:row>
     <x:row r="19" ht="76" customHeight="1">
       <x:c r="A19" s="29"/>
@@ -1884,7 +1863,6 @@
       <x:c r="F19" s="31"/>
       <x:c r="G19" s="29"/>
       <x:c r="H19" s="29"/>
-      <x:c r="I19" s="29"/>
     </x:row>
     <x:row r="20" ht="76" customHeight="1">
       <x:c r="A20" s="29"/>
@@ -1895,7 +1873,6 @@
       <x:c r="F20" s="31"/>
       <x:c r="G20" s="29"/>
       <x:c r="H20" s="29"/>
-      <x:c r="I20" s="29"/>
     </x:row>
     <x:row r="21" ht="76" customHeight="1">
       <x:c r="A21" s="29"/>
@@ -1906,7 +1883,6 @@
       <x:c r="F21" s="31"/>
       <x:c r="G21" s="29"/>
       <x:c r="H21" s="29"/>
-      <x:c r="I21" s="29"/>
     </x:row>
     <x:row r="22" ht="76" customHeight="1">
       <x:c r="A22" s="29"/>
@@ -1917,7 +1893,6 @@
       <x:c r="F22" s="31"/>
       <x:c r="G22" s="29"/>
       <x:c r="H22" s="29"/>
-      <x:c r="I22" s="29"/>
     </x:row>
     <x:row r="23" ht="76" customHeight="1">
       <x:c r="A23" s="29"/>
@@ -1928,7 +1903,6 @@
       <x:c r="F23" s="31"/>
       <x:c r="G23" s="29"/>
       <x:c r="H23" s="29"/>
-      <x:c r="I23" s="29"/>
     </x:row>
     <x:row r="24" ht="76" customHeight="1">
       <x:c r="A24" s="29"/>
@@ -1939,7 +1913,6 @@
       <x:c r="F24" s="31"/>
       <x:c r="G24" s="29"/>
       <x:c r="H24" s="29"/>
-      <x:c r="I24" s="29"/>
     </x:row>
     <x:row r="25" ht="76" customHeight="1">
       <x:c r="A25" s="29"/>
@@ -1950,7 +1923,6 @@
       <x:c r="F25" s="31"/>
       <x:c r="G25" s="29"/>
       <x:c r="H25" s="29"/>
-      <x:c r="I25" s="29"/>
     </x:row>
     <x:row r="26" ht="76" customHeight="1">
       <x:c r="A26" s="29"/>
@@ -1961,7 +1933,6 @@
       <x:c r="F26" s="31"/>
       <x:c r="G26" s="29"/>
       <x:c r="H26" s="29"/>
-      <x:c r="I26" s="29"/>
     </x:row>
     <x:row r="27" ht="76" customHeight="1">
       <x:c r="A27" s="29"/>
@@ -1972,7 +1943,6 @@
       <x:c r="F27" s="31"/>
       <x:c r="G27" s="29"/>
       <x:c r="H27" s="29"/>
-      <x:c r="I27" s="29"/>
     </x:row>
     <x:row r="28" ht="76" customHeight="1">
       <x:c r="A28" s="29"/>
@@ -1983,7 +1953,6 @@
       <x:c r="F28" s="31"/>
       <x:c r="G28" s="29"/>
       <x:c r="H28" s="29"/>
-      <x:c r="I28" s="29"/>
     </x:row>
     <x:row r="29" ht="76" customHeight="1">
       <x:c r="A29" s="29"/>
@@ -1994,7 +1963,6 @@
       <x:c r="F29" s="31"/>
       <x:c r="G29" s="29"/>
       <x:c r="H29" s="29"/>
-      <x:c r="I29" s="29"/>
     </x:row>
     <x:row r="30" ht="76" customHeight="1">
       <x:c r="A30" s="29"/>
@@ -2005,7 +1973,6 @@
       <x:c r="F30" s="31"/>
       <x:c r="G30" s="29"/>
       <x:c r="H30" s="29"/>
-      <x:c r="I30" s="29"/>
     </x:row>
     <x:row r="31" ht="76" customHeight="1">
       <x:c r="A31" s="30"/>
@@ -2016,7 +1983,6 @@
       <x:c r="F31" s="32"/>
       <x:c r="G31" s="30"/>
       <x:c r="H31" s="30"/>
-      <x:c r="I31" s="30"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">

</xml_diff>